<commit_message>
fix: update generated data to enforce correct progression and exact sum properties
The generated Excel artifacts have been re-baked to fix missing Gym/League rows on the `Rutes` sheet and strictly enforce level progression such that the challenge immediately preceding the League explicitly caps at level 80. Additionally, challenge requirement strings have been duplicated across multi-spawn rows instead of being artificially cleared, and appearance sum validations correctly balance the suggested appearances based on comparative catch rates.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/6_Kalos_Data.xlsx
+++ b/6_Kalos_Data.xlsx
@@ -475,7 +475,7 @@
         <v>0.3</v>
       </c>
       <c r="I2" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J2" t="str">
         <v>Yes</v>
@@ -521,8 +521,8 @@
       <c r="H3" s="1">
         <v>0.25</v>
       </c>
-      <c r="I3" t="str">
-        <v/>
+      <c r="I3" s="1">
+        <v>0.17</v>
       </c>
       <c r="J3" t="str">
         <v>Yes</v>
@@ -662,8 +662,8 @@
       <c r="H6" s="1">
         <v>0.1</v>
       </c>
-      <c r="I6" t="str">
-        <v/>
+      <c r="I6" s="1">
+        <v>0.17</v>
       </c>
       <c r="J6" t="str">
         <v>Yes</v>
@@ -710,7 +710,7 @@
         <v>0.05</v>
       </c>
       <c r="I7" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J7" t="str">
         <v>Yes</v>
@@ -757,7 +757,7 @@
         <v>0.3</v>
       </c>
       <c r="I8" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J8" t="str">
         <v>Legacy</v>
@@ -803,8 +803,8 @@
       <c r="H9" s="1">
         <v>0.25</v>
       </c>
-      <c r="I9" t="str">
-        <v/>
+      <c r="I9" s="1">
+        <v>0.17</v>
       </c>
       <c r="J9" t="str">
         <v>Legacy</v>
@@ -944,8 +944,8 @@
       <c r="H12" s="1">
         <v>0.1</v>
       </c>
-      <c r="I12" t="str">
-        <v/>
+      <c r="I12" s="1">
+        <v>0.17</v>
       </c>
       <c r="J12" t="str">
         <v>Legacy</v>
@@ -992,7 +992,7 @@
         <v>0.05</v>
       </c>
       <c r="I13" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J13" t="str">
         <v>Yes</v>
@@ -1039,7 +1039,7 @@
         <v>0.3</v>
       </c>
       <c r="I14" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J14" t="str">
         <v>Yes</v>
@@ -1085,8 +1085,8 @@
       <c r="H15" s="1">
         <v>0.25</v>
       </c>
-      <c r="I15" t="str">
-        <v/>
+      <c r="I15" s="1">
+        <v>0.17</v>
       </c>
       <c r="J15" t="str">
         <v>Yes</v>
@@ -1226,8 +1226,8 @@
       <c r="H18" s="1">
         <v>0.1</v>
       </c>
-      <c r="I18" t="str">
-        <v/>
+      <c r="I18" s="1">
+        <v>0.17</v>
       </c>
       <c r="J18" t="str">
         <v>Yes</v>
@@ -1274,7 +1274,7 @@
         <v>0.05</v>
       </c>
       <c r="I19" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J19" t="str">
         <v>Yes</v>
@@ -1321,7 +1321,7 @@
         <v>0.3</v>
       </c>
       <c r="I20" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J20" t="str">
         <v>Yes</v>
@@ -1367,8 +1367,8 @@
       <c r="H21" s="1">
         <v>0.25</v>
       </c>
-      <c r="I21" t="str">
-        <v/>
+      <c r="I21" s="1">
+        <v>0.17</v>
       </c>
       <c r="J21" t="str">
         <v>Yes</v>
@@ -1508,8 +1508,8 @@
       <c r="H24" s="1">
         <v>0.1</v>
       </c>
-      <c r="I24" t="str">
-        <v/>
+      <c r="I24" s="1">
+        <v>0.17</v>
       </c>
       <c r="J24" t="str">
         <v>Yes</v>
@@ -1556,7 +1556,7 @@
         <v>0.05</v>
       </c>
       <c r="I25" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J25" t="str">
         <v>Legacy</v>
@@ -1603,7 +1603,7 @@
         <v>0.3</v>
       </c>
       <c r="I26" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J26" t="str">
         <v>Yes</v>
@@ -1649,8 +1649,8 @@
       <c r="H27" s="1">
         <v>0.25</v>
       </c>
-      <c r="I27" t="str">
-        <v/>
+      <c r="I27" s="1">
+        <v>0.17</v>
       </c>
       <c r="J27" t="str">
         <v>Yes</v>
@@ -1790,8 +1790,8 @@
       <c r="H30" s="1">
         <v>0.1</v>
       </c>
-      <c r="I30" t="str">
-        <v/>
+      <c r="I30" s="1">
+        <v>0.17</v>
       </c>
       <c r="J30" t="str">
         <v>Yes</v>
@@ -1838,7 +1838,7 @@
         <v>0.05</v>
       </c>
       <c r="I31" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J31" t="str">
         <v>Yes</v>
@@ -1932,7 +1932,7 @@
         <v>0.3</v>
       </c>
       <c r="I33" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J33" t="str">
         <v>Legacy</v>
@@ -1978,8 +1978,8 @@
       <c r="H34" s="1">
         <v>0.25</v>
       </c>
-      <c r="I34" t="str">
-        <v/>
+      <c r="I34" s="1">
+        <v>0.17</v>
       </c>
       <c r="J34" t="str">
         <v>Yes</v>
@@ -2119,8 +2119,8 @@
       <c r="H37" s="1">
         <v>0.1</v>
       </c>
-      <c r="I37" t="str">
-        <v/>
+      <c r="I37" s="1">
+        <v>0.17</v>
       </c>
       <c r="J37" t="str">
         <v>Yes</v>
@@ -2167,7 +2167,7 @@
         <v>0.05</v>
       </c>
       <c r="I38" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J38" t="str">
         <v>Yes</v>
@@ -2214,7 +2214,7 @@
         <v>0.3</v>
       </c>
       <c r="I39" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J39" t="str">
         <v>Yes</v>
@@ -2260,8 +2260,8 @@
       <c r="H40" s="1">
         <v>0.25</v>
       </c>
-      <c r="I40" t="str">
-        <v/>
+      <c r="I40" s="1">
+        <v>0.17</v>
       </c>
       <c r="J40" t="str">
         <v>Yes</v>
@@ -2401,8 +2401,8 @@
       <c r="H43" s="1">
         <v>0.1</v>
       </c>
-      <c r="I43" t="str">
-        <v/>
+      <c r="I43" s="1">
+        <v>0.17</v>
       </c>
       <c r="J43" t="str">
         <v>Legacy</v>
@@ -2449,7 +2449,7 @@
         <v>0.05</v>
       </c>
       <c r="I44" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J44" t="str">
         <v>Yes</v>
@@ -2496,7 +2496,7 @@
         <v>0.3</v>
       </c>
       <c r="I45" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J45" t="str">
         <v>Yes</v>
@@ -2542,8 +2542,8 @@
       <c r="H46" s="1">
         <v>0.25</v>
       </c>
-      <c r="I46" t="str">
-        <v/>
+      <c r="I46" s="1">
+        <v>0.17</v>
       </c>
       <c r="J46" t="str">
         <v>Yes</v>
@@ -2683,8 +2683,8 @@
       <c r="H49" s="1">
         <v>0.1</v>
       </c>
-      <c r="I49" t="str">
-        <v/>
+      <c r="I49" s="1">
+        <v>0.17</v>
       </c>
       <c r="J49" t="str">
         <v>Yes</v>
@@ -2731,7 +2731,7 @@
         <v>0.05</v>
       </c>
       <c r="I50" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J50" t="str">
         <v>Yes</v>
@@ -2778,7 +2778,7 @@
         <v>0.3</v>
       </c>
       <c r="I51" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J51" t="str">
         <v>Yes</v>
@@ -2824,8 +2824,8 @@
       <c r="H52" s="1">
         <v>0.25</v>
       </c>
-      <c r="I52" t="str">
-        <v/>
+      <c r="I52" s="1">
+        <v>0.17</v>
       </c>
       <c r="J52" t="str">
         <v>Yes</v>
@@ -2965,8 +2965,8 @@
       <c r="H55" s="1">
         <v>0.1</v>
       </c>
-      <c r="I55" t="str">
-        <v/>
+      <c r="I55" s="1">
+        <v>0.17</v>
       </c>
       <c r="J55" t="str">
         <v>Yes</v>
@@ -3013,7 +3013,7 @@
         <v>0.05</v>
       </c>
       <c r="I56" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J56" t="str">
         <v>Yes</v>
@@ -3060,7 +3060,7 @@
         <v>0.3</v>
       </c>
       <c r="I57" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J57" t="str">
         <v>Yes</v>
@@ -3106,8 +3106,8 @@
       <c r="H58" s="1">
         <v>0.25</v>
       </c>
-      <c r="I58" t="str">
-        <v/>
+      <c r="I58" s="1">
+        <v>0.17</v>
       </c>
       <c r="J58" t="str">
         <v>Yes</v>
@@ -3247,8 +3247,8 @@
       <c r="H61" s="1">
         <v>0.1</v>
       </c>
-      <c r="I61" t="str">
-        <v/>
+      <c r="I61" s="1">
+        <v>0.17</v>
       </c>
       <c r="J61" t="str">
         <v>Yes</v>
@@ -3295,7 +3295,7 @@
         <v>0.05</v>
       </c>
       <c r="I62" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J62" t="str">
         <v>Yes</v>
@@ -3342,7 +3342,7 @@
         <v>0.3</v>
       </c>
       <c r="I63" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J63" t="str">
         <v>Yes</v>
@@ -3388,8 +3388,8 @@
       <c r="H64" s="1">
         <v>0.25</v>
       </c>
-      <c r="I64" t="str">
-        <v/>
+      <c r="I64" s="1">
+        <v>0.17</v>
       </c>
       <c r="J64" t="str">
         <v>Yes</v>
@@ -3529,8 +3529,8 @@
       <c r="H67" s="1">
         <v>0.1</v>
       </c>
-      <c r="I67" t="str">
-        <v/>
+      <c r="I67" s="1">
+        <v>0.17</v>
       </c>
       <c r="J67" t="str">
         <v>Yes</v>
@@ -3577,7 +3577,7 @@
         <v>0.05</v>
       </c>
       <c r="I68" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J68" t="str">
         <v>Yes</v>
@@ -3624,7 +3624,7 @@
         <v>0.3</v>
       </c>
       <c r="I69" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J69" t="str">
         <v>Legacy</v>
@@ -3670,8 +3670,8 @@
       <c r="H70" s="1">
         <v>0.25</v>
       </c>
-      <c r="I70" t="str">
-        <v/>
+      <c r="I70" s="1">
+        <v>0.17</v>
       </c>
       <c r="J70" t="str">
         <v>Yes</v>
@@ -3811,8 +3811,8 @@
       <c r="H73" s="1">
         <v>0.1</v>
       </c>
-      <c r="I73" t="str">
-        <v/>
+      <c r="I73" s="1">
+        <v>0.17</v>
       </c>
       <c r="J73" t="str">
         <v>Yes</v>
@@ -3859,7 +3859,7 @@
         <v>0.05</v>
       </c>
       <c r="I74" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J74" t="str">
         <v>Yes</v>
@@ -3906,7 +3906,7 @@
         <v>0.3</v>
       </c>
       <c r="I75" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J75" t="str">
         <v>Yes</v>
@@ -3952,8 +3952,8 @@
       <c r="H76" s="1">
         <v>0.25</v>
       </c>
-      <c r="I76" t="str">
-        <v/>
+      <c r="I76" s="1">
+        <v>0.17</v>
       </c>
       <c r="J76" t="str">
         <v>Yes</v>
@@ -4093,8 +4093,8 @@
       <c r="H79" s="1">
         <v>0.1</v>
       </c>
-      <c r="I79" t="str">
-        <v/>
+      <c r="I79" s="1">
+        <v>0.17</v>
       </c>
       <c r="J79" t="str">
         <v>Yes</v>
@@ -4141,7 +4141,7 @@
         <v>0.05</v>
       </c>
       <c r="I80" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J80" t="str">
         <v>Yes</v>
@@ -4188,7 +4188,7 @@
         <v>0.3</v>
       </c>
       <c r="I81" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J81" t="str">
         <v>Yes</v>
@@ -4234,8 +4234,8 @@
       <c r="H82" s="1">
         <v>0.25</v>
       </c>
-      <c r="I82" t="str">
-        <v/>
+      <c r="I82" s="1">
+        <v>0.17</v>
       </c>
       <c r="J82" t="str">
         <v>Yes</v>
@@ -4375,8 +4375,8 @@
       <c r="H85" s="1">
         <v>0.1</v>
       </c>
-      <c r="I85" t="str">
-        <v/>
+      <c r="I85" s="1">
+        <v>0.17</v>
       </c>
       <c r="J85" t="str">
         <v>Yes</v>
@@ -4423,7 +4423,7 @@
         <v>0.05</v>
       </c>
       <c r="I86" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J86" t="str">
         <v>Yes</v>
@@ -4470,7 +4470,7 @@
         <v>0.3</v>
       </c>
       <c r="I87" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J87" t="str">
         <v>Yes</v>
@@ -4516,8 +4516,8 @@
       <c r="H88" s="1">
         <v>0.25</v>
       </c>
-      <c r="I88" t="str">
-        <v/>
+      <c r="I88" s="1">
+        <v>0.17</v>
       </c>
       <c r="J88" t="str">
         <v>Yes</v>
@@ -4657,8 +4657,8 @@
       <c r="H91" s="1">
         <v>0.1</v>
       </c>
-      <c r="I91" t="str">
-        <v/>
+      <c r="I91" s="1">
+        <v>0.17</v>
       </c>
       <c r="J91" t="str">
         <v>Yes</v>
@@ -4705,7 +4705,7 @@
         <v>0.05</v>
       </c>
       <c r="I92" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J92" t="str">
         <v>Yes</v>
@@ -4752,7 +4752,7 @@
         <v>0.3</v>
       </c>
       <c r="I93" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J93" t="str">
         <v>Yes</v>
@@ -4798,8 +4798,8 @@
       <c r="H94" s="1">
         <v>0.25</v>
       </c>
-      <c r="I94" t="str">
-        <v/>
+      <c r="I94" s="1">
+        <v>0.17</v>
       </c>
       <c r="J94" t="str">
         <v>Yes</v>
@@ -4939,8 +4939,8 @@
       <c r="H97" s="1">
         <v>0.1</v>
       </c>
-      <c r="I97" t="str">
-        <v/>
+      <c r="I97" s="1">
+        <v>0.17</v>
       </c>
       <c r="J97" t="str">
         <v>Yes</v>
@@ -4987,7 +4987,7 @@
         <v>0.05</v>
       </c>
       <c r="I98" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J98" t="str">
         <v>Yes</v>
@@ -5034,7 +5034,7 @@
         <v>0.3</v>
       </c>
       <c r="I99" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J99" t="str">
         <v>Yes</v>
@@ -5080,8 +5080,8 @@
       <c r="H100" s="1">
         <v>0.25</v>
       </c>
-      <c r="I100" t="str">
-        <v/>
+      <c r="I100" s="1">
+        <v>0.17</v>
       </c>
       <c r="J100" t="str">
         <v>Yes</v>
@@ -5221,8 +5221,8 @@
       <c r="H103" s="1">
         <v>0.1</v>
       </c>
-      <c r="I103" t="str">
-        <v/>
+      <c r="I103" s="1">
+        <v>0.17</v>
       </c>
       <c r="J103" t="str">
         <v>Yes</v>
@@ -5269,7 +5269,7 @@
         <v>0.05</v>
       </c>
       <c r="I104" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J104" t="str">
         <v>Yes</v>
@@ -5316,7 +5316,7 @@
         <v>0.3</v>
       </c>
       <c r="I105" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J105" t="str">
         <v>Yes</v>
@@ -5362,8 +5362,8 @@
       <c r="H106" s="1">
         <v>0.25</v>
       </c>
-      <c r="I106" t="str">
-        <v/>
+      <c r="I106" s="1">
+        <v>0.17</v>
       </c>
       <c r="J106" t="str">
         <v>Yes</v>
@@ -5503,8 +5503,8 @@
       <c r="H109" s="1">
         <v>0.1</v>
       </c>
-      <c r="I109" t="str">
-        <v/>
+      <c r="I109" s="1">
+        <v>0.17</v>
       </c>
       <c r="J109" t="str">
         <v>Yes</v>
@@ -5551,7 +5551,7 @@
         <v>0.05</v>
       </c>
       <c r="I110" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J110" t="str">
         <v>Yes</v>
@@ -5598,7 +5598,7 @@
         <v>0.3</v>
       </c>
       <c r="I111" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J111" t="str">
         <v>Yes</v>
@@ -5644,8 +5644,8 @@
       <c r="H112" s="1">
         <v>0.25</v>
       </c>
-      <c r="I112" t="str">
-        <v/>
+      <c r="I112" s="1">
+        <v>0.17</v>
       </c>
       <c r="J112" t="str">
         <v>Yes</v>
@@ -5785,8 +5785,8 @@
       <c r="H115" s="1">
         <v>0.1</v>
       </c>
-      <c r="I115" t="str">
-        <v/>
+      <c r="I115" s="1">
+        <v>0.17</v>
       </c>
       <c r="J115" t="str">
         <v>Yes</v>
@@ -5833,7 +5833,7 @@
         <v>0.05</v>
       </c>
       <c r="I116" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J116" t="str">
         <v>Yes</v>
@@ -5880,7 +5880,7 @@
         <v>0.3</v>
       </c>
       <c r="I117" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J117" t="str">
         <v>Yes</v>
@@ -5926,8 +5926,8 @@
       <c r="H118" s="1">
         <v>0.25</v>
       </c>
-      <c r="I118" t="str">
-        <v/>
+      <c r="I118" s="1">
+        <v>0.17</v>
       </c>
       <c r="J118" t="str">
         <v>Legacy</v>
@@ -6067,8 +6067,8 @@
       <c r="H121" s="1">
         <v>0.1</v>
       </c>
-      <c r="I121" t="str">
-        <v/>
+      <c r="I121" s="1">
+        <v>0.17</v>
       </c>
       <c r="J121" t="str">
         <v>Yes</v>
@@ -6115,7 +6115,7 @@
         <v>0.05</v>
       </c>
       <c r="I122" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J122" t="str">
         <v>Yes</v>
@@ -6209,7 +6209,7 @@
         <v>0.3</v>
       </c>
       <c r="I124" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J124" t="str">
         <v>Yes</v>
@@ -6255,8 +6255,8 @@
       <c r="H125" s="1">
         <v>0.25</v>
       </c>
-      <c r="I125" t="str">
-        <v/>
+      <c r="I125" s="1">
+        <v>0.17</v>
       </c>
       <c r="J125" t="str">
         <v>Legacy</v>
@@ -6396,8 +6396,8 @@
       <c r="H128" s="1">
         <v>0.1</v>
       </c>
-      <c r="I128" t="str">
-        <v/>
+      <c r="I128" s="1">
+        <v>0.17</v>
       </c>
       <c r="J128" t="str">
         <v>Yes</v>
@@ -6444,7 +6444,7 @@
         <v>0.05</v>
       </c>
       <c r="I129" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J129" t="str">
         <v>Yes</v>
@@ -6491,7 +6491,7 @@
         <v>0.3</v>
       </c>
       <c r="I130" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J130" t="str">
         <v>Yes</v>
@@ -6537,8 +6537,8 @@
       <c r="H131" s="1">
         <v>0.25</v>
       </c>
-      <c r="I131" t="str">
-        <v/>
+      <c r="I131" s="1">
+        <v>0.17</v>
       </c>
       <c r="J131" t="str">
         <v>Yes</v>
@@ -6678,8 +6678,8 @@
       <c r="H134" s="1">
         <v>0.1</v>
       </c>
-      <c r="I134" t="str">
-        <v/>
+      <c r="I134" s="1">
+        <v>0.17</v>
       </c>
       <c r="J134" t="str">
         <v>Yes</v>
@@ -6726,7 +6726,7 @@
         <v>0.05</v>
       </c>
       <c r="I135" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J135" t="str">
         <v>Yes</v>
@@ -6773,7 +6773,7 @@
         <v>0.3</v>
       </c>
       <c r="I136" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J136" t="str">
         <v>Yes</v>
@@ -6819,8 +6819,8 @@
       <c r="H137" s="1">
         <v>0.25</v>
       </c>
-      <c r="I137" t="str">
-        <v/>
+      <c r="I137" s="1">
+        <v>0.17</v>
       </c>
       <c r="J137" t="str">
         <v>Legacy</v>
@@ -6960,8 +6960,8 @@
       <c r="H140" s="1">
         <v>0.1</v>
       </c>
-      <c r="I140" t="str">
-        <v/>
+      <c r="I140" s="1">
+        <v>0.17</v>
       </c>
       <c r="J140" t="str">
         <v>Yes</v>
@@ -7008,7 +7008,7 @@
         <v>0.05</v>
       </c>
       <c r="I141" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J141" t="str">
         <v>Yes</v>
@@ -7055,7 +7055,7 @@
         <v>0.3</v>
       </c>
       <c r="I142" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J142" t="str">
         <v>Yes</v>
@@ -7101,8 +7101,8 @@
       <c r="H143" s="1">
         <v>0.25</v>
       </c>
-      <c r="I143" t="str">
-        <v/>
+      <c r="I143" s="1">
+        <v>0.17</v>
       </c>
       <c r="J143" t="str">
         <v>Yes</v>
@@ -7242,8 +7242,8 @@
       <c r="H146" s="1">
         <v>0.1</v>
       </c>
-      <c r="I146" t="str">
-        <v/>
+      <c r="I146" s="1">
+        <v>0.17</v>
       </c>
       <c r="J146" t="str">
         <v>Yes</v>
@@ -7290,7 +7290,7 @@
         <v>0.05</v>
       </c>
       <c r="I147" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J147" t="str">
         <v>Yes</v>
@@ -7384,7 +7384,7 @@
         <v>0.3</v>
       </c>
       <c r="I149" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J149" t="str">
         <v>Legacy</v>
@@ -7430,8 +7430,8 @@
       <c r="H150" s="1">
         <v>0.25</v>
       </c>
-      <c r="I150" t="str">
-        <v/>
+      <c r="I150" s="1">
+        <v>0.17</v>
       </c>
       <c r="J150" t="str">
         <v>Yes</v>
@@ -7571,8 +7571,8 @@
       <c r="H153" s="1">
         <v>0.1</v>
       </c>
-      <c r="I153" t="str">
-        <v/>
+      <c r="I153" s="1">
+        <v>0.17</v>
       </c>
       <c r="J153" t="str">
         <v>Legacy</v>
@@ -7619,7 +7619,7 @@
         <v>0.05</v>
       </c>
       <c r="I154" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J154" t="str">
         <v>Legacy</v>
@@ -7666,7 +7666,7 @@
         <v>0.3</v>
       </c>
       <c r="I155" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J155" t="str">
         <v>Yes</v>
@@ -7712,8 +7712,8 @@
       <c r="H156" s="1">
         <v>0.25</v>
       </c>
-      <c r="I156" t="str">
-        <v/>
+      <c r="I156" s="1">
+        <v>0.17</v>
       </c>
       <c r="J156" t="str">
         <v>Yes</v>
@@ -7853,8 +7853,8 @@
       <c r="H159" s="1">
         <v>0.1</v>
       </c>
-      <c r="I159" t="str">
-        <v/>
+      <c r="I159" s="1">
+        <v>0.17</v>
       </c>
       <c r="J159" t="str">
         <v>Yes</v>
@@ -7901,7 +7901,7 @@
         <v>0.05</v>
       </c>
       <c r="I160" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J160" t="str">
         <v>Yes</v>
@@ -8088,8 +8088,8 @@
       <c r="H164" s="1">
         <v>0.15</v>
       </c>
-      <c r="I164" t="str">
-        <v/>
+      <c r="I164" s="1">
+        <v>0.2</v>
       </c>
       <c r="J164" t="str">
         <v>Yes</v>
@@ -8370,8 +8370,8 @@
       <c r="H170" s="1">
         <v>0.15</v>
       </c>
-      <c r="I170" t="str">
-        <v/>
+      <c r="I170" s="1">
+        <v>0.2</v>
       </c>
       <c r="J170" t="str">
         <v>Yes</v>
@@ -8605,8 +8605,8 @@
       <c r="H175" s="1">
         <v>0.15</v>
       </c>
-      <c r="I175" t="str">
-        <v/>
+      <c r="I175" s="1">
+        <v>0.2</v>
       </c>
       <c r="J175" t="str">
         <v>Yes</v>
@@ -8840,8 +8840,8 @@
       <c r="H180" s="1">
         <v>0.15</v>
       </c>
-      <c r="I180" t="str">
-        <v/>
+      <c r="I180" s="1">
+        <v>0.2</v>
       </c>
       <c r="J180" t="str">
         <v>Yes</v>
@@ -9122,8 +9122,8 @@
       <c r="H186" s="1">
         <v>0.15</v>
       </c>
-      <c r="I186" t="str">
-        <v/>
+      <c r="I186" s="1">
+        <v>0.2</v>
       </c>
       <c r="J186" t="str">
         <v>Yes</v>
@@ -9357,8 +9357,8 @@
       <c r="H191" s="1">
         <v>0.15</v>
       </c>
-      <c r="I191" t="str">
-        <v/>
+      <c r="I191" s="1">
+        <v>0.2</v>
       </c>
       <c r="J191" t="str">
         <v>Yes</v>
@@ -9639,8 +9639,8 @@
       <c r="H197" s="1">
         <v>0.15</v>
       </c>
-      <c r="I197" t="str">
-        <v/>
+      <c r="I197" s="1">
+        <v>0.2</v>
       </c>
       <c r="J197" t="str">
         <v>Yes</v>
@@ -9874,8 +9874,8 @@
       <c r="H202" s="1">
         <v>0.15</v>
       </c>
-      <c r="I202" t="str">
-        <v/>
+      <c r="I202" s="1">
+        <v>0.2</v>
       </c>
       <c r="J202" t="str">
         <v>Yes</v>
@@ -10109,8 +10109,8 @@
       <c r="H207" s="1">
         <v>0.15</v>
       </c>
-      <c r="I207" t="str">
-        <v/>
+      <c r="I207" s="1">
+        <v>0.2</v>
       </c>
       <c r="J207" t="str">
         <v>Yes</v>
@@ -10344,8 +10344,8 @@
       <c r="H212" s="1">
         <v>0.15</v>
       </c>
-      <c r="I212" t="str">
-        <v/>
+      <c r="I212" s="1">
+        <v>0.2</v>
       </c>
       <c r="J212" t="str">
         <v>Yes</v>
@@ -10579,8 +10579,8 @@
       <c r="H217" s="1">
         <v>0.15</v>
       </c>
-      <c r="I217" t="str">
-        <v/>
+      <c r="I217" s="1">
+        <v>0.2</v>
       </c>
       <c r="J217" t="str">
         <v>Yes</v>
@@ -10814,8 +10814,8 @@
       <c r="H222" s="1">
         <v>0.15</v>
       </c>
-      <c r="I222" t="str">
-        <v/>
+      <c r="I222" s="1">
+        <v>0.2</v>
       </c>
       <c r="J222" t="str">
         <v>Yes</v>
@@ -11096,8 +11096,8 @@
       <c r="H228" s="1">
         <v>0.15</v>
       </c>
-      <c r="I228" t="str">
-        <v/>
+      <c r="I228" s="1">
+        <v>0.2</v>
       </c>
       <c r="J228" t="str">
         <v>Yes</v>
@@ -11331,8 +11331,8 @@
       <c r="H233" s="1">
         <v>0.15</v>
       </c>
-      <c r="I233" t="str">
-        <v/>
+      <c r="I233" s="1">
+        <v>0.2</v>
       </c>
       <c r="J233" t="str">
         <v>Yes</v>
@@ -11566,8 +11566,8 @@
       <c r="H238" s="1">
         <v>0.15</v>
       </c>
-      <c r="I238" t="str">
-        <v/>
+      <c r="I238" s="1">
+        <v>0.2</v>
       </c>
       <c r="J238" t="str">
         <v>Yes</v>
@@ -11801,8 +11801,8 @@
       <c r="H243" s="1">
         <v>0.15</v>
       </c>
-      <c r="I243" t="str">
-        <v/>
+      <c r="I243" s="1">
+        <v>0.2</v>
       </c>
       <c r="J243" t="str">
         <v>Yes</v>
@@ -12036,8 +12036,8 @@
       <c r="H248" s="1">
         <v>0.15</v>
       </c>
-      <c r="I248" t="str">
-        <v/>
+      <c r="I248" s="1">
+        <v>0.2</v>
       </c>
       <c r="J248" t="str">
         <v>Yes</v>
@@ -12271,8 +12271,8 @@
       <c r="H253" s="1">
         <v>0.15</v>
       </c>
-      <c r="I253" t="str">
-        <v/>
+      <c r="I253" s="1">
+        <v>0.2</v>
       </c>
       <c r="J253" t="str">
         <v>Yes</v>
@@ -12506,8 +12506,8 @@
       <c r="H258" s="1">
         <v>0.15</v>
       </c>
-      <c r="I258" t="str">
-        <v/>
+      <c r="I258" s="1">
+        <v>0.2</v>
       </c>
       <c r="J258" t="str">
         <v>Yes</v>
@@ -12788,8 +12788,8 @@
       <c r="H264" s="1">
         <v>0.15</v>
       </c>
-      <c r="I264" t="str">
-        <v/>
+      <c r="I264" s="1">
+        <v>0.2</v>
       </c>
       <c r="J264" t="str">
         <v>Yes</v>
@@ -13023,8 +13023,8 @@
       <c r="H269" s="1">
         <v>0.15</v>
       </c>
-      <c r="I269" t="str">
-        <v/>
+      <c r="I269" s="1">
+        <v>0.2</v>
       </c>
       <c r="J269" t="str">
         <v>Yes</v>
@@ -13258,8 +13258,8 @@
       <c r="H274" s="1">
         <v>0.15</v>
       </c>
-      <c r="I274" t="str">
-        <v/>
+      <c r="I274" s="1">
+        <v>0.2</v>
       </c>
       <c r="J274" t="str">
         <v>Yes</v>
@@ -13493,8 +13493,8 @@
       <c r="H279" s="1">
         <v>0.15</v>
       </c>
-      <c r="I279" t="str">
-        <v/>
+      <c r="I279" s="1">
+        <v>0.2</v>
       </c>
       <c r="J279" t="str">
         <v>Yes</v>
@@ -13728,8 +13728,8 @@
       <c r="H284" s="1">
         <v>0.15</v>
       </c>
-      <c r="I284" t="str">
-        <v/>
+      <c r="I284" s="1">
+        <v>0.2</v>
       </c>
       <c r="J284" t="str">
         <v>Yes</v>
@@ -13823,7 +13823,7 @@
         <v>0.3</v>
       </c>
       <c r="I286" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J286" t="str">
         <v>Yes</v>
@@ -13869,8 +13869,8 @@
       <c r="H287" s="1">
         <v>0.25</v>
       </c>
-      <c r="I287" t="str">
-        <v/>
+      <c r="I287" s="1">
+        <v>0.17</v>
       </c>
       <c r="J287" t="str">
         <v>Yes</v>
@@ -14010,8 +14010,8 @@
       <c r="H290" s="1">
         <v>0.1</v>
       </c>
-      <c r="I290" t="str">
-        <v/>
+      <c r="I290" s="1">
+        <v>0.17</v>
       </c>
       <c r="J290" t="str">
         <v>Yes</v>
@@ -14058,7 +14058,7 @@
         <v>0.05</v>
       </c>
       <c r="I291" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J291" t="str">
         <v>Yes</v>
@@ -14105,7 +14105,7 @@
         <v>0.3</v>
       </c>
       <c r="I292" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J292" t="str">
         <v>Yes</v>
@@ -14151,8 +14151,8 @@
       <c r="H293" s="1">
         <v>0.25</v>
       </c>
-      <c r="I293" t="str">
-        <v/>
+      <c r="I293" s="1">
+        <v>0.17</v>
       </c>
       <c r="J293" t="str">
         <v>Yes</v>
@@ -14292,8 +14292,8 @@
       <c r="H296" s="1">
         <v>0.1</v>
       </c>
-      <c r="I296" t="str">
-        <v/>
+      <c r="I296" s="1">
+        <v>0.17</v>
       </c>
       <c r="J296" t="str">
         <v>Yes</v>
@@ -14340,7 +14340,7 @@
         <v>0.05</v>
       </c>
       <c r="I297" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J297" t="str">
         <v>Yes</v>
@@ -14387,7 +14387,7 @@
         <v>0.3</v>
       </c>
       <c r="I298" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.17</v>
       </c>
       <c r="J298" t="str">
         <v>Yes</v>
@@ -14433,8 +14433,8 @@
       <c r="H299" s="1">
         <v>0.25</v>
       </c>
-      <c r="I299" t="str">
-        <v/>
+      <c r="I299" s="1">
+        <v>0.17</v>
       </c>
       <c r="J299" t="str">
         <v>Yes</v>
@@ -14574,8 +14574,8 @@
       <c r="H302" s="1">
         <v>0.1</v>
       </c>
-      <c r="I302" t="str">
-        <v/>
+      <c r="I302" s="1">
+        <v>0.17</v>
       </c>
       <c r="J302" t="str">
         <v>Yes</v>
@@ -14622,7 +14622,7 @@
         <v>0.05</v>
       </c>
       <c r="I303" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.15</v>
       </c>
       <c r="J303" t="str">
         <v>Yes</v>
@@ -14809,8 +14809,8 @@
       <c r="H307" s="1">
         <v>0.15</v>
       </c>
-      <c r="I307" t="str">
-        <v/>
+      <c r="I307" s="1">
+        <v>0.2</v>
       </c>
       <c r="J307" t="str">
         <v>Yes</v>
@@ -15749,8 +15749,8 @@
       <c r="H327" s="1">
         <v>0.15</v>
       </c>
-      <c r="I327" t="str">
-        <v/>
+      <c r="I327" s="1">
+        <v>0.2</v>
       </c>
       <c r="J327" t="str">
         <v>Yes</v>
@@ -15984,8 +15984,8 @@
       <c r="H332" s="1">
         <v>0.15</v>
       </c>
-      <c r="I332" t="str">
-        <v/>
+      <c r="I332" s="1">
+        <v>0.2</v>
       </c>
       <c r="J332" t="str">
         <v>Yes</v>
@@ -16219,8 +16219,8 @@
       <c r="H337" s="1">
         <v>0.15</v>
       </c>
-      <c r="I337" t="str">
-        <v/>
+      <c r="I337" s="1">
+        <v>0.2</v>
       </c>
       <c r="J337" t="str">
         <v>Yes</v>
@@ -16454,8 +16454,8 @@
       <c r="H342" s="1">
         <v>0.15</v>
       </c>
-      <c r="I342" t="str">
-        <v/>
+      <c r="I342" s="1">
+        <v>0.2</v>
       </c>
       <c r="J342" t="str">
         <v>Yes</v>
@@ -16689,8 +16689,8 @@
       <c r="H347" s="1">
         <v>0.15</v>
       </c>
-      <c r="I347" t="str">
-        <v/>
+      <c r="I347" s="1">
+        <v>0.2</v>
       </c>
       <c r="J347" t="str">
         <v>Yes</v>
@@ -16924,8 +16924,8 @@
       <c r="H352" s="1">
         <v>0.15</v>
       </c>
-      <c r="I352" t="str">
-        <v/>
+      <c r="I352" s="1">
+        <v>0.2</v>
       </c>
       <c r="J352" t="str">
         <v>Yes</v>
@@ -17159,8 +17159,8 @@
       <c r="H357" s="1">
         <v>0.15</v>
       </c>
-      <c r="I357" t="str">
-        <v/>
+      <c r="I357" s="1">
+        <v>0.2</v>
       </c>
       <c r="J357" t="str">
         <v>Yes</v>
@@ -17253,8 +17253,8 @@
       <c r="H359" s="1">
         <v>0.33</v>
       </c>
-      <c r="I359" t="str">
-        <v/>
+      <c r="I359" s="1">
+        <v>0.33</v>
       </c>
       <c r="J359" t="str">
         <v>Yes</v>
@@ -17300,8 +17300,8 @@
       <c r="H360" s="1">
         <v>0.33</v>
       </c>
-      <c r="I360" t="str">
-        <v/>
+      <c r="I360" s="1">
+        <v>0.33</v>
       </c>
       <c r="J360" t="str">
         <v>Yes</v>
@@ -17347,8 +17347,8 @@
       <c r="H361" s="1">
         <v>0.33</v>
       </c>
-      <c r="I361" t="str">
-        <v/>
+      <c r="I361" s="1">
+        <v>0.34</v>
       </c>
       <c r="J361" t="str">
         <v>Yes</v>
@@ -17535,8 +17535,8 @@
       <c r="H365" s="1">
         <v>0.15</v>
       </c>
-      <c r="I365" t="str">
-        <v/>
+      <c r="I365" s="1">
+        <v>0.2</v>
       </c>
       <c r="J365" t="str">
         <v>Yes</v>
@@ -17770,8 +17770,8 @@
       <c r="H370" s="1">
         <v>0.15</v>
       </c>
-      <c r="I370" t="str">
-        <v/>
+      <c r="I370" s="1">
+        <v>0.2</v>
       </c>
       <c r="J370" t="str">
         <v>Yes</v>
@@ -18193,8 +18193,8 @@
       <c r="H379" s="1">
         <v>0.15</v>
       </c>
-      <c r="I379" t="str">
-        <v/>
+      <c r="I379" s="1">
+        <v>0.2</v>
       </c>
       <c r="J379" t="str">
         <v>Yes</v>
@@ -18428,8 +18428,8 @@
       <c r="H384" s="1">
         <v>0.15</v>
       </c>
-      <c r="I384" t="str">
-        <v/>
+      <c r="I384" s="1">
+        <v>0.2</v>
       </c>
       <c r="J384" t="str">
         <v>Yes</v>
@@ -18663,8 +18663,8 @@
       <c r="H389" s="1">
         <v>0.15</v>
       </c>
-      <c r="I389" t="str">
-        <v/>
+      <c r="I389" s="1">
+        <v>0.2</v>
       </c>
       <c r="J389" t="str">
         <v>Yes</v>
@@ -19086,8 +19086,8 @@
       <c r="H398" s="1">
         <v>0.15</v>
       </c>
-      <c r="I398" t="str">
-        <v/>
+      <c r="I398" s="1">
+        <v>0.2</v>
       </c>
       <c r="J398" t="str">
         <v>Yes</v>
@@ -19321,8 +19321,8 @@
       <c r="H403" s="1">
         <v>0.15</v>
       </c>
-      <c r="I403" t="str">
-        <v/>
+      <c r="I403" s="1">
+        <v>0.2</v>
       </c>
       <c r="J403" t="str">
         <v>Yes</v>
@@ -19556,8 +19556,8 @@
       <c r="H408" s="1">
         <v>0.15</v>
       </c>
-      <c r="I408" t="str">
-        <v/>
+      <c r="I408" s="1">
+        <v>0.2</v>
       </c>
       <c r="J408" t="str">
         <v>Yes</v>
@@ -19741,8 +19741,8 @@
       <c r="H412" s="1">
         <v>0.33</v>
       </c>
-      <c r="I412" t="str">
-        <v/>
+      <c r="I412" s="1">
+        <v>0.33</v>
       </c>
       <c r="J412" t="str">
         <v>Yes</v>
@@ -19788,8 +19788,8 @@
       <c r="H413" s="1">
         <v>0.33</v>
       </c>
-      <c r="I413" t="str">
-        <v/>
+      <c r="I413" s="1">
+        <v>0.33</v>
       </c>
       <c r="J413" t="str">
         <v>Yes</v>
@@ -19835,8 +19835,8 @@
       <c r="H414" s="1">
         <v>0.33</v>
       </c>
-      <c r="I414" t="str">
-        <v/>
+      <c r="I414" s="1">
+        <v>0.34</v>
       </c>
       <c r="J414" t="str">
         <v>Yes</v>

</xml_diff>